<commit_message>
Switch to xlwriter. Clean up context md files.
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/sample-data/sample-run/selections/Ultimates.xlsx
+++ b/sample-data/sample-run/selections/Ultimates.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Losses" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,9 +26,20 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -41,26 +51,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDE7F6"/>
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE6CC"/>
+        <fgColor rgb="FFF4B084"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -68,46 +82,33 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -473,22 +474,12 @@
   <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="18.7109375" customWidth="1" min="1" max="11"/>
+    <col width="30.7109375" customWidth="1" min="12" max="12"/>
+    <col width="18.7109375" customWidth="1" min="13" max="13"/>
+    <col width="30.7109375" customWidth="1" min="14" max="14"/>
+    <col width="18.7109375" customWidth="1" min="15" max="15"/>
+    <col width="40.7109375" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -611,21 +602,21 @@
       <c r="K2" s="4" t="n">
         <v>3054159.61</v>
       </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>Paid Loss selected. Paid CL ultimate of 3,054,159.61. Year is at extreme tail maturity (287 months, 100% developed). Incurred IE disqualified (negative IBNR -121,479). Paid CL is primary method for fully-developed tail periods; closure rate stable (CDF 1.0039). Convergence not applicable—Paid CL is sole viable method at this age.</t>
-        </is>
-      </c>
-      <c r="M2" s="6" t="n">
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Paid Loss selected. Paid CL ultimate of 3,054,159.61. Year is at extreme tail maturity (287 months, 100% developed). Incurred IE disqualified (negative IBNR -121,479). Paid CL is primary method for fully-developed tail periods; closure rate stable (CDF 1.0039). Convergence not applicableâ€”Paid CL is sole viable method at this age.</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="n">
         <v>3054159.61</v>
       </c>
-      <c r="N2" s="7" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Fully mature (287 months); Paid and Incurred ultimates nearly converge. Paid preferred for stability; CL ultimate of 3,054,160 is credible with minimal IBNR (11,865).</t>
         </is>
       </c>
-      <c r="O2" s="8" t="n"/>
-      <c r="P2" s="9" t="n"/>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -665,21 +656,21 @@
       <c r="K3" s="4" t="n">
         <v>2216836.93</v>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 2,216,836.93. Age 275 months, 99.2% developed. Incurred IE disqualified (negative IBNR -704,698). Paid CL is standard for tail years. Paid development very stable (CDF 1.0078). Incurred CL secondary (2,406,196.57) but Paid CL preferred at this extreme maturity.</t>
         </is>
       </c>
-      <c r="M3" s="6" t="n">
+      <c r="M3" s="5" t="n">
         <v>2216836.93</v>
       </c>
-      <c r="N3" s="7" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Mature (275 months, 99% developed); Incurred shows high estimate (2,904,344) with negative IBNR bias. Paid CL of 2,216,837 aligns with economic patterns; low IBNR of 17,191.</t>
         </is>
       </c>
-      <c r="O3" s="8" t="n"/>
-      <c r="P3" s="9" t="n"/>
+      <c r="O3" s="6" t="n"/>
+      <c r="P3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -719,21 +710,21 @@
       <c r="K4" s="4" t="n">
         <v>1805248.44</v>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 1,805,248.44. Age 263 months (&gt;20 years). Incurred IE disqualified (negative IBNR -855,180). Paid CL (1,805,248.44) vs. Incurred CL (1,838,027.15): difference 1.8%. Paid CL preferred for tail maturity with stable closure rate (CDF 1.0153).</t>
         </is>
       </c>
-      <c r="M4" s="6" t="n">
+      <c r="M4" s="5" t="n">
         <v>1805248.44</v>
       </c>
-      <c r="N4" s="7" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Mature (263 months, 98% developed); Incurred at 1,838,027 vs Paid at 1,805,248. Paid CL of 1,805,248 preferred for stability; Incurred shows IBNR of 59,936 suggesting conservative estimate in tail.</t>
         </is>
       </c>
-      <c r="O4" s="8" t="n"/>
-      <c r="P4" s="9" t="n"/>
+      <c r="O4" s="6" t="n"/>
+      <c r="P4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -773,21 +764,21 @@
       <c r="K5" s="4" t="n">
         <v>1146826.99</v>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 1,146,826.99. Age 251 months. Incurred IE disqualified (negative IBNR -556,096). Paid CL (1,146,826.99) vs. Incurred CL (1,180,647.54): 2.9% difference. Paid CL is primary for late tail; stable closure dynamics (CDF 1.0216).</t>
         </is>
       </c>
-      <c r="M5" s="6" t="n">
+      <c r="M5" s="5" t="n">
         <v>1146826.99</v>
       </c>
-      <c r="N5" s="7" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Mature (251 months, 98% developed); Paid CL of 1,146,827 slightly below Incurred CL of 1,180,648. Paid preferred for lower tail volatility; IBNR of 24,212 is modest.</t>
         </is>
       </c>
-      <c r="O5" s="8" t="n"/>
-      <c r="P5" s="9" t="n"/>
+      <c r="O5" s="6" t="n"/>
+      <c r="P5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -827,21 +818,21 @@
       <c r="K6" s="4" t="n">
         <v>2302875.95</v>
       </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 2,302,875.95. Age 239 months. Incurred IE disqualified (negative IBNR of -529,863 is implausible; case adequacy assumption broken). Paid CL (2,302,875.95) vs. Incurred CL (2,374,326.11): 3.0% difference. Paid CL preferred for stability; Incurred methods unreliable.</t>
         </is>
       </c>
-      <c r="M6" s="6" t="n">
+      <c r="M6" s="5" t="n">
         <v>2302875.95</v>
       </c>
-      <c r="N6" s="7" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Mature (239 months, 94% developed); Incurred shows negative IBNR (-529,864), indicating overstatement in prior periods. Paid CL of 2,302,876 is credible with positive IBNR of 60,727.</t>
         </is>
       </c>
-      <c r="O6" s="8" t="n"/>
-      <c r="P6" s="9" t="n"/>
+      <c r="O6" s="6" t="n"/>
+      <c r="P6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -881,21 +872,21 @@
       <c r="K7" s="4" t="n">
         <v>1505496.3</v>
       </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 1,505,496.30. Age 227 months (late tail). Incurred IE disqualified (negative IBNR -284,389). Paid CL (1,505,496.30) vs. Incurred CL (1,621,406.24): 7.1% difference. Paid CL preferred; Incurred CL link ratios show instability (case adequacy shifting). Paid development stable (CDF 1.0297).</t>
         </is>
       </c>
-      <c r="M7" s="6" t="n">
+      <c r="M7" s="5" t="n">
         <v>1505496.3</v>
       </c>
-      <c r="N7" s="7" t="inlineStr">
+      <c r="N7" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Mature (227 months, 97% developed); Incurred at 1,621,406 and Paid at 1,505,496 diverge moderately. Paid CL of 1,505,496 preferred given cleaner paid emergence; positive IBNR of 43,355.</t>
         </is>
       </c>
-      <c r="O7" s="8" t="n"/>
-      <c r="P7" s="9" t="n"/>
+      <c r="O7" s="6" t="n"/>
+      <c r="P7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -935,21 +926,21 @@
       <c r="K8" s="4" t="n">
         <v>4955930.27</v>
       </c>
-      <c r="L8" s="5" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 4,955,930.27. Age 215 months. Incurred IE disqualified (negative IBNR of -1,960,436; case adequacy severely degraded). Paid CL (4,955,930.27) vs. Incurred CL (5,139,714.61): 3.6% difference. Paid CL preferred; Incurred methods unreliable due to case reserve instability. Paid CDF 1.0345 is reasonable.</t>
         </is>
       </c>
-      <c r="M8" s="6" t="n">
+      <c r="M8" s="5" t="n">
         <v>4955930.27</v>
       </c>
-      <c r="N8" s="7" t="inlineStr">
+      <c r="N8" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Mature (215 months, 97% developed); Incurred shows negative IBNR (-1,960,436) reflecting volatility in incurred reporting. Paid CL of 4,955,930 is stable; IBNR of 165,237 reasonable for 97% developed.</t>
         </is>
       </c>
-      <c r="O8" s="8" t="n"/>
-      <c r="P8" s="9" t="n"/>
+      <c r="O8" s="6" t="n"/>
+      <c r="P8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -989,21 +980,21 @@
       <c r="K9" s="4" t="n">
         <v>1428966.22</v>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 1,428,966.22. Age 203 months. Incurred IE disqualified (negative IBNR -1,165,499). Paid CL (1,428,966.22) vs. Incurred CL (1,475,624.25): 3.2% difference. Paid CL is stable; Incurred CL shows case adequacy issues (CDF 1.0705). Paid development is more credible (CDF 1.0367).</t>
         </is>
       </c>
-      <c r="M9" s="6" t="n">
+      <c r="M9" s="5" t="n">
         <v>1428966.22</v>
       </c>
-      <c r="N9" s="7" t="inlineStr">
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Mature (203 months, 96% developed); Incurred inflated estimate (2,543,927) with IBNR of 1,165,499 appears inconsistent with development pattern. Paid CL of 1,428,966 with IBNR of 50,538 more credible.</t>
         </is>
       </c>
-      <c r="O9" s="8" t="n"/>
-      <c r="P9" s="9" t="n"/>
+      <c r="O9" s="6" t="n"/>
+      <c r="P9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1043,21 +1034,21 @@
       <c r="K10" s="4" t="n">
         <v>1226405.58</v>
       </c>
-      <c r="L10" s="5" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 1,226,405.58. Age 191 months. Incurred IE disqualified (negative IBNR -1,425,224). Paid CL (1,226,405.58) vs. Incurred CL (1,261,566.69): 2.8% difference. Paid CL preferred; Incurred CL link ratios unstable (CDF 1.0786 vs. Paid CDF 1.0486). Paid method more credible.</t>
         </is>
       </c>
-      <c r="M10" s="6" t="n">
+      <c r="M10" s="5" t="n">
         <v>1226405.58</v>
       </c>
-      <c r="N10" s="7" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Mature (191 months, 95% developed); Incurred at 2,594,806 with huge IBNR (1,425,225) seems excessive given maturity. Paid CL of 1,226,406 with moderate IBNR of 56,824 more reasonable.</t>
         </is>
       </c>
-      <c r="O10" s="8" t="n"/>
-      <c r="P10" s="9" t="n"/>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1097,21 +1088,21 @@
       <c r="K11" s="4" t="n">
         <v>1360648.28</v>
       </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 1,360,648.28. Age 179 months. Incurred IE disqualified (negative IBNR of -143,371; case adequacy assumption violated). Paid CL (1,360,648.28) vs. Incurred CL (1,383,120.22): 1.6% difference within convergence band. Paid CL selected; closure rate stable (CDF 1.0649) and Paid method more robust.</t>
         </is>
       </c>
-      <c r="M11" s="6" t="n">
+      <c r="M11" s="5" t="n">
         <v>1360648.28</v>
       </c>
-      <c r="N11" s="7" t="inlineStr">
+      <c r="N11" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Mature (179 months, 94% developed); Incurred shows negative IBNR (-143,371) suggesting overestimation in prior reporting. Paid CL of 1,360,648 is stable with reasonable IBNR of 82,976.</t>
         </is>
       </c>
-      <c r="O11" s="8" t="n"/>
-      <c r="P11" s="9" t="n"/>
+      <c r="O11" s="6" t="n"/>
+      <c r="P11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1151,21 +1142,21 @@
       <c r="K12" s="4" t="n">
         <v>2044396.42</v>
       </c>
-      <c r="L12" s="5" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 2,044,396.42. Age 167 months. Incurred IE disqualified (negative IBNR of -373,432). Paid CL (2,044,396.42) vs. Incurred CL (2,117,984.61): 3.5% difference. Paid CL preferred; Incurred CL shows elevated CDF (1.1054) indicating link ratio volatility and case reserve degradation. Paid development more stable (CDF 1.0802).</t>
         </is>
       </c>
-      <c r="M12" s="6" t="n">
+      <c r="M12" s="5" t="n">
         <v>2044396.42</v>
       </c>
-      <c r="N12" s="7" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Semi-mature (167 months, 93% developed); Incurred at 2,117,985 vs Paid at 2,044,396. Paid CL of 2,044,396 preferred; IBNR of 151,738 reasonable given development level.</t>
         </is>
       </c>
-      <c r="O12" s="8" t="n"/>
-      <c r="P12" s="9" t="n"/>
+      <c r="O12" s="6" t="n"/>
+      <c r="P12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1205,21 +1196,21 @@
       <c r="K13" s="4" t="n">
         <v>1307266.94</v>
       </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>Paid Loss selected. Paid CL ultimate of 1,307,266.94. Age 155 months (late maturity, 60–84 months band lower range). Incurred IE disqualified (negative IBNR -209,748). Paid CL (1,307,266.94) vs. Incurred CL (1,508,058.98): 13.3% divergence signals Incurred CL instability. Paid CL is primary; closure rate stable (CDF 1.0946).</t>
-        </is>
-      </c>
-      <c r="M13" s="6" t="n">
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Paid Loss selected. Paid CL ultimate of 1,307,266.94. Age 155 months (late maturity, 60â€“84 months band lower range). Incurred IE disqualified (negative IBNR -209,748). Paid CL (1,307,266.94) vs. Incurred CL (1,508,058.98): 13.3% divergence signals Incurred CL instability. Paid CL is primary; closure rate stable (CDF 1.0946).</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="n">
         <v>1307266.94</v>
       </c>
-      <c r="N13" s="7" t="inlineStr">
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Semi-mature (155 months, 91% developed); Incurred shows positive IBNR but higher estimate (1,508,059). Paid CL of 1,307,267 is stable baseline; IBNR of 113,030 proportional to development.</t>
         </is>
       </c>
-      <c r="O13" s="8" t="n"/>
-      <c r="P13" s="9" t="n"/>
+      <c r="O13" s="6" t="n"/>
+      <c r="P13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1259,21 +1250,21 @@
       <c r="K14" s="4" t="n">
         <v>789162.53</v>
       </c>
-      <c r="L14" s="5" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 789,162.53. Age 143 months. Incurred IE disqualified (negative IBNR -495,199). Paid CL (789,162.53) vs. Incurred CL (785,226.82): 0.5% convergence within acceptable band. Paid CL selected; both methods close but Paid shows superior fitness (stable CDF 1.1138 vs. Incurred CDF 1.0823 suggests CDF escalation anomaly in Incurred). Paid preferred.</t>
         </is>
       </c>
-      <c r="M14" s="6" t="n">
+      <c r="M14" s="5" t="n">
         <v>789162.53</v>
       </c>
-      <c r="N14" s="7" t="inlineStr">
+      <c r="N14" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Semi-mature (143 months, 90% developed); Incurred at 785,227 vs Paid at 789,163 converge closely. Paid CL of 789,163 slightly higher but within method variance; IBNR of 80,633.</t>
         </is>
       </c>
-      <c r="O14" s="8" t="n"/>
-      <c r="P14" s="9" t="n"/>
+      <c r="O14" s="6" t="n"/>
+      <c r="P14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1313,21 +1304,21 @@
       <c r="K15" s="4" t="n">
         <v>1576996.53</v>
       </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 1,576,996.53. Age 131 months (late-to-mid transition, 84 months threshold). Incurred IE disqualified (negative IBNR of -161,800). Paid CL (1,576,996.53) vs. Incurred CL (1,593,926.14): 1.1% convergence. Paid CL selected; late maturity band and Paid method's stability preferred. CDF 1.1349 shows development still present.</t>
         </is>
       </c>
-      <c r="M15" s="6" t="n">
+      <c r="M15" s="5" t="n">
         <v>1576996.53</v>
       </c>
-      <c r="N15" s="7" t="inlineStr">
+      <c r="N15" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Semi-mature (131 months, 88% developed); Incurred at 1,593,926 slightly higher. Paid CL of 1,576,997 represents stable development with reasonable IBNR of 187,393 given maturity.</t>
         </is>
       </c>
-      <c r="O15" s="8" t="n"/>
-      <c r="P15" s="9" t="n"/>
+      <c r="O15" s="6" t="n"/>
+      <c r="P15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1367,21 +1358,21 @@
       <c r="K16" s="4" t="n">
         <v>3849598.12</v>
       </c>
-      <c r="L16" s="5" t="inlineStr">
+      <c r="L16" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 3,849,598.12. Age 119 months (mid-maturity band). Incurred IE disqualified (negative IBNR of -1,713,150; implausible). Paid CL (3,849,598.12) vs. Incurred CL (3,912,201.44): 1.6% convergence. Paid CL selected; Incurred IE severely disqualified, and Paid CL stability preferred at this maturity. CDF 1.1443 indicates meaningful development remains.</t>
         </is>
       </c>
-      <c r="M16" s="6" t="n">
+      <c r="M16" s="5" t="n">
         <v>3849598.12</v>
       </c>
-      <c r="N16" s="7" t="inlineStr">
+      <c r="N16" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Semi-mature (119 months, 87% developed); Incurred shows negative IBNR (-1,713,150) reflecting reporting volatility. Paid CL of 3,849,598 with IBNR of 485,367 more credible given 87% development.</t>
         </is>
       </c>
-      <c r="O16" s="8" t="n"/>
-      <c r="P16" s="9" t="n"/>
+      <c r="O16" s="6" t="n"/>
+      <c r="P16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1421,21 +1412,21 @@
       <c r="K17" s="4" t="n">
         <v>2999163</v>
       </c>
-      <c r="L17" s="5" t="inlineStr">
-        <is>
-          <t>Paid Loss selected. Paid CL ultimate of 2,999,163.00. Age 107 months (mid-maturity, 60–84 month band). Incurred IE disqualified (negative IBNR -48,490 marginal). Paid CL (2,999,163.00) vs. Incurred CL (3,038,991.70): 1.3% convergence. Paid CL selected; entering mid-maturity phase where Paid CL remains primary. CDF 1.2181 shows substantial development ahead.</t>
-        </is>
-      </c>
-      <c r="M17" s="6" t="n">
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Paid Loss selected. Paid CL ultimate of 2,999,163.00. Age 107 months (mid-maturity, 60â€“84 month band). Incurred IE disqualified (negative IBNR -48,490 marginal). Paid CL (2,999,163.00) vs. Incurred CL (3,038,991.70): 1.3% convergence. Paid CL selected; entering mid-maturity phase where Paid CL remains primary. CDF 1.2181 shows substantial development ahead.</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="n">
         <v>2999163</v>
       </c>
-      <c r="N17" s="7" t="inlineStr">
+      <c r="N17" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Semi-mature (107 months, 82% developed); Incurred at 3,038,992 vs Paid at 2,999,163. Paid CL of 2,999,163 preferred; methods generally converge; IBNR of 536,954 appropriate for 82% maturity.</t>
         </is>
       </c>
-      <c r="O17" s="8" t="n"/>
-      <c r="P17" s="9" t="n"/>
+      <c r="O17" s="6" t="n"/>
+      <c r="P17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1475,21 +1466,21 @@
       <c r="K18" s="4" t="n">
         <v>1488161.05</v>
       </c>
-      <c r="L18" s="5" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 1,488,161.05. Age 95 months (mid-maturity lower range). Incurred IE disqualified (negative IBNR -1,400,098; implausible). Paid CL (1,488,161.05) vs. Incurred CL (1,483,428.99): 0.3% convergence. Both very close; Paid CL selected for superior fitness. CDF 1.2342 indicates ~19% development remaining.</t>
         </is>
       </c>
-      <c r="M18" s="6" t="n">
+      <c r="M18" s="5" t="n">
         <v>1488161.05</v>
       </c>
-      <c r="N18" s="7" t="inlineStr">
+      <c r="N18" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Developing (95 months, 81% developed); Incurred shows large IBNR (277,617) with high tail factor (CDF 1.230). Paid CL of 1,488,161 more stable; IBNR of 282,349 reasonable for development stage.</t>
         </is>
       </c>
-      <c r="O18" s="8" t="n"/>
-      <c r="P18" s="9" t="n"/>
+      <c r="O18" s="6" t="n"/>
+      <c r="P18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1529,21 +1520,21 @@
       <c r="K19" s="4" t="n">
         <v>3053327.91</v>
       </c>
-      <c r="L19" s="5" t="inlineStr">
-        <is>
-          <t>Paid Loss selected. Paid CL ultimate of 3,053,327.91. Age 83 months (mid-maturity band, 36–60+ mo). Incurred IE disqualified (negative IBNR of -180,424). Paid CL (3,053,327.91) vs. Incurred CL (2,966,113.90): 2.9% difference. Paid CL selected; Incurred IE failure disqualifies blending. CDF 1.2746 shows significant development. Paid method more robust at this maturity.</t>
-        </is>
-      </c>
-      <c r="M19" s="6" t="n">
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Paid Loss selected. Paid CL ultimate of 3,053,327.91. Age 83 months (mid-maturity band, 36â€“60+ mo). Incurred IE disqualified (negative IBNR of -180,424). Paid CL (3,053,327.91) vs. Incurred CL (2,966,113.90): 2.9% difference. Paid CL selected; Incurred IE failure disqualifies blending. CDF 1.2746 shows significant development. Paid method more robust at this maturity.</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="n">
         <v>3053327.91</v>
       </c>
-      <c r="N19" s="7" t="inlineStr">
+      <c r="N19" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Developing (83 months, 78% developed); Incurred shows negative IBNR (-180,425) despite high CDF. Paid CL of 3,053,328 with IBNR of 657,879 reflects consistent development; tail factor CDF 1.275.</t>
         </is>
       </c>
-      <c r="O19" s="8" t="n"/>
-      <c r="P19" s="9" t="n"/>
+      <c r="O19" s="6" t="n"/>
+      <c r="P19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1583,21 +1574,21 @@
       <c r="K20" s="4" t="n">
         <v>3379669.12</v>
       </c>
-      <c r="L20" s="5" t="inlineStr">
-        <is>
-          <t>Paid Loss selected. Paid CL ultimate of 3,379,669.12. Age 71 months (early maturity, 36–60 boundary). Incurred IE disqualified (negative IBNR of -340,558). Paid CL (3,379,669.12) vs. Incurred CL (3,499,325.39): 3.4% difference. Paid CL selected; ~29% development remains (CDF 1.4110). At early maturity, Paid CL credibility exceeds Incurred CL; Incurred IE disqualified.</t>
-        </is>
-      </c>
-      <c r="M20" s="6" t="n">
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Paid Loss selected. Paid CL ultimate of 3,379,669.12. Age 71 months (early maturity, 36â€“60 boundary). Incurred IE disqualified (negative IBNR of -340,558). Paid CL (3,379,669.12) vs. Incurred CL (3,499,325.39): 3.4% difference. Paid CL selected; ~29% development remains (CDF 1.4110). At early maturity, Paid CL credibility exceeds Incurred CL; Incurred IE disqualified.</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="n">
         <v>3379669.12</v>
       </c>
-      <c r="N20" s="7" t="inlineStr">
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Developing (71 months, 71% developed); Paid CL of 3,379,669 with IBNR of 984,479 is stable anchor. Incurred shows negative IBNR (-340,559) inconsistent with development pattern. Paid CDF of 1.411 appropriate for maturity.</t>
         </is>
       </c>
-      <c r="O20" s="8" t="n"/>
-      <c r="P20" s="9" t="n"/>
+      <c r="O20" s="6" t="n"/>
+      <c r="P20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1637,21 +1628,21 @@
       <c r="K21" s="4" t="n">
         <v>1541396.59</v>
       </c>
-      <c r="L21" s="5" t="inlineStr">
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 1,541,396.59. Age 59 months (early maturity, high immaturity). Incurred IE disqualified (negative IBNR -864,708). Paid CL (1,541,396.59) vs. Incurred CL (1,452,867.57): 5.8% divergence signals Incurred instability. Paid CL is primary; ~37% development remains (CDF 1.5792). Paid BF secondary (1,652,240.31) is 7.2% higher but Paid CL credible at 59 months.</t>
         </is>
       </c>
-      <c r="M21" s="6" t="n">
+      <c r="M21" s="5" t="n">
         <v>1541396.59</v>
       </c>
-      <c r="N21" s="7" t="inlineStr">
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Early developing (59 months, 63% developed); Paid CL of 1,541,397 with IBNR of 565,346 reflects early development stage. CDF of 1.579 substantial but credible given only 63% maturity. Incurred at 1,452,867 lower, but Paid CL more stable.</t>
         </is>
       </c>
-      <c r="O21" s="8" t="n"/>
-      <c r="P21" s="9" t="n"/>
+      <c r="O21" s="6" t="n"/>
+      <c r="P21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1691,21 +1682,21 @@
       <c r="K22" s="4" t="n">
         <v>1690287.65</v>
       </c>
-      <c r="L22" s="5" t="inlineStr">
-        <is>
-          <t>Paid Loss selected. Paid CL ultimate of 1,690,287.65. Age 47 months (green maturity, 24–36 boundary). Incurred IE disqualified (negative IBNR -435,380). Paid CL (1,690,287.65) vs. Incurred CL (1,586,080.90): 6.2% divergence. At green maturity, baseline is BF-heavy, but Paid CL (1,690,287.65) and Paid BF (1,571,825.99) differ 7.0%. Paid CL selected as more data-driven; 42% development remains (CDF 1.7337).</t>
-        </is>
-      </c>
-      <c r="M22" s="6" t="n">
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Paid Loss selected. Paid CL ultimate of 1,690,287.65. Age 47 months (green maturity, 24â€“36 boundary). Incurred IE disqualified (negative IBNR -435,380). Paid CL (1,690,287.65) vs. Incurred CL (1,586,080.90): 6.2% divergence. At green maturity, baseline is BF-heavy, but Paid CL (1,690,287.65) and Paid BF (1,571,825.99) differ 7.0%. Paid CL selected as more data-driven; 42% development remains (CDF 1.7337).</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="n">
         <v>1690287.65</v>
       </c>
-      <c r="N22" s="7" t="inlineStr">
+      <c r="N22" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Early developing (47 months, 58% developed); Paid CL of 1,690,288 with IBNR of 715,308 reflects 58% development. CDF of 1.734 reflects high tail uncertainty. Incurred at 1,586,081 lower but Paid CL provides more conservative tail estimate.</t>
         </is>
       </c>
-      <c r="O22" s="8" t="n"/>
-      <c r="P22" s="9" t="n"/>
+      <c r="O22" s="6" t="n"/>
+      <c r="P22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1745,21 +1736,21 @@
       <c r="K23" s="4" t="n">
         <v>1645673.39</v>
       </c>
-      <c r="L23" s="5" t="inlineStr">
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid CL ultimate of 1,645,673.39. Age 35 months (green, transitioning toward very green). Paid CL (1,645,673.39) vs. Paid BF (1,289,119.20): 21.6% divergence signals extreme immaturity. Paid BF is typically primary for &lt;24 mo. However, ~52% development has occurred (CDF 2.0802). Paid CL selected with reduced confidence due to potential link ratio volatility; Incurred IE disqualified (negative IBNR -167,941).</t>
         </is>
       </c>
-      <c r="M23" s="6" t="n">
+      <c r="M23" s="5" t="n">
         <v>1645673.39</v>
       </c>
-      <c r="N23" s="7" t="inlineStr">
+      <c r="N23" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Early developing (35 months, 48% developed); Paid CL of 1,645,673 with IBNR of 854,570 reflects 48% development stage and high uncertainty (CDF 2.080). Incurred at 1,557,461 lower but tail factor higher at 1.882; Paid CL more stable.</t>
         </is>
       </c>
-      <c r="O23" s="8" t="n"/>
-      <c r="P23" s="9" t="n"/>
+      <c r="O23" s="6" t="n"/>
+      <c r="P23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1799,21 +1790,21 @@
       <c r="K24" s="4" t="n">
         <v>1846864.71</v>
       </c>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>Paid Loss selected. Paid BF ultimate of 1,846,864.71. Age 23 months (very green, 12–24 month boundary). Paid CL (3,548,451.09) shows extreme elevation (CDF 2.9589, 66% development) indicating volatile link ratios at extreme immaturity. Paid BF (1,846,864.71) is more stable method for very early years; prior loss ratio credible. Incurred IE disqualified (negative IBNR of -221,016). Paid BF is primary at this age.</t>
-        </is>
-      </c>
-      <c r="M24" s="6" t="n">
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Paid Loss selected. Paid BF ultimate of 1,846,864.71. Age 23 months (very green, 12â€“24 month boundary). Paid CL (3,548,451.09) shows extreme elevation (CDF 2.9589, 66% development) indicating volatile link ratios at extreme immaturity. Paid BF (1,846,864.71) is more stable method for very early years; prior loss ratio credible. Incurred IE disqualified (negative IBNR of -221,016). Paid BF is primary at this age.</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="n">
         <v>3548451.09</v>
       </c>
-      <c r="N24" s="7" t="inlineStr">
+      <c r="N24" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Immature (23 months, 34% developed); Paid CL of 3,548,451 with high IBNR of 2,349,209 reflects substantial development ahead (CDF 2.959). Incurred at 3,909,735 higher with lower IBNR, but Paid CL more consistent with tail development pattern.</t>
         </is>
       </c>
-      <c r="O24" s="8" t="n"/>
-      <c r="P24" s="9" t="n"/>
+      <c r="O24" s="6" t="n"/>
+      <c r="P24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1853,25 +1844,25 @@
       <c r="K25" s="4" t="n">
         <v>1224487.09</v>
       </c>
-      <c r="L25" s="5" t="inlineStr">
+      <c r="L25" s="4" t="inlineStr">
         <is>
           <t>Paid Loss selected. Paid BF ultimate of 1,224,487.09. Age 11 months (&lt;12 months, extreme immaturity). Paid CL (2,757,367.94) inflated by extreme CDF (7.7618) indicating unreliable link ratios (&lt;13% developed). Paid BF (1,224,487.09) is primary method for a priori estimation at extreme youth; prior loss ratio informative. Incurred IE disqualified (negative IBNR -642,542). Paid BF selected per maturity-based hierarchy for very green years.</t>
         </is>
       </c>
-      <c r="M25" s="6" t="n">
+      <c r="M25" s="5" t="n">
         <v>2757367.94</v>
       </c>
-      <c r="N25" s="7" t="inlineStr">
+      <c r="N25" s="5" t="inlineStr">
         <is>
           <t>Paid Loss, Chain Ladder. Highly immature (11 months, 13% developed); Paid CL of 2,757,368 with extreme IBNR of 2,402,120 reflects very early stage (CDF 7.762). High uncertainty but CL is most credible single-method selection given maturity constraints and paid emergence patterns.</t>
         </is>
       </c>
-      <c r="O25" s="8" t="n"/>
-      <c r="P25" s="9" t="n"/>
+      <c r="O25" s="6" t="n"/>
+      <c r="P25" s="6" t="n"/>
     </row>
     <row r="26"/>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1884,18 +1875,12 @@
   <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="18.7109375" customWidth="1" min="1" max="7"/>
+    <col width="30.7109375" customWidth="1" min="8" max="8"/>
+    <col width="18.7109375" customWidth="1" min="9" max="9"/>
+    <col width="30.7109375" customWidth="1" min="10" max="10"/>
+    <col width="18.7109375" customWidth="1" min="11" max="11"/>
+    <col width="40.7109375" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1986,21 +1971,21 @@
       <c r="G2" s="4" t="n">
         <v>700.71</v>
       </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>Reported Count selected. Reported CL ultimate of 700.71 (CDF 1.0, 100% developed). All methods (CL, IE, BF) converge at 700.7–700.8 for fully-developed tail period. Reported IE (700.78) is 0.01% higher but adds minimal IBNR (0.07 counts). Reported CL selected as standard method for fully-developed years. Count data shows no case adequacy issues.</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="n">
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Reported Count selected. Reported CL ultimate of 700.71 (CDF 1.0, 100% developed). All methods (CL, IE, BF) converge at 700.7â€“700.8 for fully-developed tail period. Reported IE (700.78) is 0.01% higher but adds minimal IBNR (0.07 counts). Reported CL selected as standard method for fully-developed years. Count data shows no case adequacy issues.</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="n">
         <v>700.71</v>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 287 months); all methods converge at 700.71. No IBNR needed; count development complete.</t>
         </is>
       </c>
-      <c r="K2" s="8" t="n"/>
-      <c r="L2" s="9" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2028,21 +2013,21 @@
       <c r="G3" s="4" t="n">
         <v>651.88</v>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 651.88 (CDF 1.0, 100% developed). Reported IE (683.17) shows elevated IBNR (+31.28 counts), implying late reporting, but at full maturity this is implausible. Reported CL is primary. Reported BF (651.88) identical. Selection based on data-driven CL at extreme tail maturity.</t>
         </is>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I3" s="5" t="n">
         <v>651.88</v>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 275 months); CL ultimate of 651.88 with zero IBNR. IE method (683.17) and BF method (651.88) converge on same estimate.</t>
         </is>
       </c>
-      <c r="K3" s="8" t="n"/>
-      <c r="L3" s="9" t="n"/>
+      <c r="K3" s="6" t="n"/>
+      <c r="L3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2070,21 +2055,21 @@
       <c r="G4" s="4" t="n">
         <v>551.59</v>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 551.59 (CDF 1.0, 100% developed). Reported IE projects 648.44 (+96.85 IBNR) but this contradicts full development; case adequacy assumption fails. Reported CL is sole credible method at full maturity. IE disqualified due to implausible late reporting assumption at 100% development.</t>
         </is>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="I4" s="5" t="n">
         <v>551.59</v>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 263 months); CL ultimate of 551.59. IE suggests higher estimate (648.44) with positive IBNR of 96.85; CL preferred for fully developed year.</t>
         </is>
       </c>
-      <c r="K4" s="8" t="n"/>
-      <c r="L4" s="9" t="n"/>
+      <c r="K4" s="6" t="n"/>
+      <c r="L4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2112,21 +2097,21 @@
       <c r="G5" s="4" t="n">
         <v>642.65</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 642.65 (CDF 1.0, 100% developed). Reported IE (627.84) shows negative IBNR (-14.81), disqualifying it. Reported BF (642.65) identical. Reported CL is primary. Count is fully developed; no late-reporting signal.</t>
         </is>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="5" t="n">
         <v>642.65</v>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 251 months); CL ultimate of 642.65 with zero IBNR. IE method shows negative IBNR (-14.81) suggesting reported count is stable and complete.</t>
         </is>
       </c>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="9" t="n"/>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2154,21 +2139,21 @@
       <c r="G6" s="4" t="n">
         <v>641.33</v>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 641.33 (CDF 1.0, 100% developed). Reported IE (623.61) shows negative IBNR (-17.71), disqualifying case adequacy assumption. Reported BF (641.33) identical. CL is standard at full maturity; IE fitness fails.</t>
         </is>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I6" s="5" t="n">
         <v>641.33</v>
       </c>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 239 months); CL ultimate of 641.33. IE and BF converge at similar levels; reported count development is complete.</t>
         </is>
       </c>
-      <c r="K6" s="8" t="n"/>
-      <c r="L6" s="9" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2196,21 +2181,21 @@
       <c r="G7" s="4" t="n">
         <v>497.49</v>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 497.49 (CDF 1.0, 100% developed). Reported IE (606.74) projects +109.26 IBNR despite full development; assumption violated. Reported BF (497.49) identical. Reported CL is sole credible method at maturity level.</t>
         </is>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I7" s="5" t="n">
         <v>497.49</v>
       </c>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 227 months); CL ultimate of 497.49. IE method estimates 606.74 with large IBNR (109.26), but CL is credible for fully developed year.</t>
         </is>
       </c>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="9" t="n"/>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2238,21 +2223,21 @@
       <c r="G8" s="4" t="n">
         <v>476.38</v>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 476.38 (CDF 1.0, 100% developed). Reported IE (550.47) shows +74.10 IBNR; implausible at full development. Reported CL is primary. IE disqualified. BF matches CL.</t>
         </is>
       </c>
-      <c r="I8" s="6" t="n">
+      <c r="I8" s="5" t="n">
         <v>476.38</v>
       </c>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 215 months); CL ultimate of 476.38. IE method shows inflation (550.47) with IBNR of 74.10; CL preferred for fully matured cohort.</t>
         </is>
       </c>
-      <c r="K8" s="8" t="n"/>
-      <c r="L8" s="9" t="n"/>
+      <c r="K8" s="6" t="n"/>
+      <c r="L8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2280,21 +2265,21 @@
       <c r="G9" s="4" t="n">
         <v>328.58</v>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 328.58 (CDF 1.0, 100% developed). Reported IE (444.10) projects +115.52 IBNR despite full maturity; case adequacy assumption fails at 100% development. Reported CL is standard. IE disqualified for implausible development assumption.</t>
         </is>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="I9" s="5" t="n">
         <v>328.58</v>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 203 months); CL ultimate of 328.58. IE inflates estimate to 444.10 with IBNR of 115.52; CL more conservative and credible.</t>
         </is>
       </c>
-      <c r="K9" s="8" t="n"/>
-      <c r="L9" s="9" t="n"/>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2322,21 +2307,21 @@
       <c r="G10" s="4" t="n">
         <v>321.98</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 321.98 (CDF 1.0, 100% developed). Reported IE (384.40) shows +62.42 IBNR; implausible at full development. Reported BF (321.98) matches CL. Reported CL is primary; IE fitness fails.</t>
         </is>
       </c>
-      <c r="I10" s="6" t="n">
+      <c r="I10" s="5" t="n">
         <v>321.98</v>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 191 months); CL ultimate of 321.98. IE method (384.40) shows inflation with IBNR of 62.42; CL preferred for fully reported cohort.</t>
         </is>
       </c>
-      <c r="K10" s="8" t="n"/>
-      <c r="L10" s="9" t="n"/>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2364,21 +2349,21 @@
       <c r="G11" s="4" t="n">
         <v>271.84</v>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 271.84 (CDF 1.0, 100% developed). Reported IE (314.20) projects +42.36 IBNR despite full development; case adequacy assumption violated. Reported CL selected as standard at maturity. IE disqualified.</t>
         </is>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="I11" s="5" t="n">
         <v>271.84</v>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 179 months); CL ultimate of 271.84. IE and BF estimates higher; CL reflects actual reported count maturity.</t>
         </is>
       </c>
-      <c r="K11" s="8" t="n"/>
-      <c r="L11" s="9" t="n"/>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2406,21 +2391,21 @@
       <c r="G12" s="4" t="n">
         <v>345.74</v>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 345.74 (CDF 1.0, 100% developed). Reported IE (319.33) shows negative IBNR (-26.41), disqualifying case adequacy model. Reported BF (345.74) matches CL. CL is primary at full maturity; IE fitness fails.</t>
         </is>
       </c>
-      <c r="I12" s="6" t="n">
+      <c r="I12" s="5" t="n">
         <v>345.74</v>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 167 months); CL ultimate of 345.74. IE method shows negative IBNR (-26.41) suggesting reported counts are complete and stable.</t>
         </is>
       </c>
-      <c r="K12" s="8" t="n"/>
-      <c r="L12" s="9" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2448,21 +2433,21 @@
       <c r="G13" s="4" t="n">
         <v>261.28</v>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 261.28 (CDF 1.0, 100% developed). Reported IE (298.97) shows +37.68 IBNR despite full development; assumption violated. Reported BF (261.28) identical. Reported CL is primary. IE disqualified.</t>
         </is>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="I13" s="5" t="n">
         <v>261.28</v>
       </c>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 155 months); CL ultimate of 261.28. IE method shows IBNR of 37.68; CL is most credible for fully reported year.</t>
         </is>
       </c>
-      <c r="K13" s="8" t="n"/>
-      <c r="L13" s="9" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2490,21 +2475,21 @@
       <c r="G14" s="4" t="n">
         <v>291.63</v>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 291.63 (CDF 1.0, 100% developed). Reported IE (305.75) shows +14.12 IBNR despite full maturity; implausible. Reported BF (291.63) matches CL. Reported CL is standard at full development; IE fitness marginal but fails on plausibility.</t>
         </is>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="I14" s="5" t="n">
         <v>291.63</v>
       </c>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 143 months); CL ultimate of 291.63. Methods show modest IBNR ranges; CL is credible and centered estimate.</t>
         </is>
       </c>
-      <c r="K14" s="8" t="n"/>
-      <c r="L14" s="9" t="n"/>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2532,21 +2517,21 @@
       <c r="G15" s="4" t="n">
         <v>455.26</v>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 455.26 (CDF 1.0, 100% developed). Reported IE (341.33) shows negative IBNR (-113.93), disqualifying case adequacy assumption. Reported BF (455.26) matches CL. Reported CL is primary; IE fitness fails.</t>
         </is>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I15" s="5" t="n">
         <v>455.26</v>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 131 months); CL ultimate of 455.26. IE method shows negative IBNR (-113.93) suggesting reported counts are complete; CL is credible.</t>
         </is>
       </c>
-      <c r="K15" s="8" t="n"/>
-      <c r="L15" s="9" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2574,21 +2559,21 @@
       <c r="G16" s="4" t="n">
         <v>333.86</v>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 333.86 (CDF 1.0, 100% developed). Reported IE (367.36) shows +33.50 IBNR at full development; assumption violated. Reported BF (333.86) identical. Reported CL is standard at maturity. IE disqualified on fitness grounds.</t>
         </is>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="I16" s="5" t="n">
         <v>333.86</v>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Fully developed (CDF 1.0, 119 months); CL ultimate of 333.86. IE method shows modest IBNR of 33.50; CL represents reported count maturity.</t>
         </is>
       </c>
-      <c r="K16" s="8" t="n"/>
-      <c r="L16" s="9" t="n"/>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2616,21 +2601,21 @@
       <c r="G17" s="4" t="n">
         <v>389.7</v>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 389.70 (CDF 0.9977, 100.2% developed). Slight CDF &lt;1.0 indicates potential reopens or count adjustments (marginal). Reported IE (401.53) shows +10.93 IBNR (2.7% adjustment). Reported CL selected as primary; IE is secondary backup. BF shows minimal negative IBNR (-0.93). CL is most credible.</t>
         </is>
       </c>
-      <c r="I17" s="6" t="n">
+      <c r="I17" s="5" t="n">
         <v>389.7</v>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Nearly mature (CDF 0.9977, 107 months); CL ultimate of 389.70 with slight negative IBNR (-0.90). BF method shows similar result; development is essentially complete.</t>
         </is>
       </c>
-      <c r="K17" s="8" t="n"/>
-      <c r="L17" s="9" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2658,21 +2643,21 @@
       <c r="G18" s="4" t="n">
         <v>309.39</v>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 309.39 (CDF 0.9977, 100.2% developed). Similar to 2016, slight CDF &lt;1.0 (reopens marginal). Reported IE (351.80) shows +41.69 IBNR (13.5% inflation) despite near-full development; fitness questionable. Reported CL is primary. BF shows minor negative (-0.81). CL most credible.</t>
         </is>
       </c>
-      <c r="I18" s="6" t="n">
+      <c r="I18" s="5" t="n">
         <v>309.39</v>
       </c>
-      <c r="J18" s="7" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Nearly mature (CDF 0.9977, 95 months); CL ultimate of 309.39 with minimal IBNR (-0.71). IE method estimates 351.80 with IBNR of 41.69; CL reflects lower development tail.</t>
         </is>
       </c>
-      <c r="K18" s="8" t="n"/>
-      <c r="L18" s="9" t="n"/>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2700,21 +2685,21 @@
       <c r="G19" s="4" t="n">
         <v>324.96</v>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 324.96 (CDF 0.997, 100.3% developed). CDF &lt;1.0 indicates marginal reopens. Reported IE (349.53) shows +23.59 IBNR (7.3% adjustment); fitness marginal. Reported CL is primary for near-full development. BF shows minor negative (-1.05). CL selected.</t>
         </is>
       </c>
-      <c r="I19" s="6" t="n">
+      <c r="I19" s="5" t="n">
         <v>324.96</v>
       </c>
-      <c r="J19" s="7" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Nearly mature (CDF 0.9970, 83 months); CL ultimate of 324.96 with slight negative IBNR (-0.98). IE and BF show slightly higher estimates; CL credible for near-mature cohort.</t>
         </is>
       </c>
-      <c r="K19" s="8" t="n"/>
-      <c r="L19" s="9" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2742,21 +2727,21 @@
       <c r="G20" s="4" t="n">
         <v>356.54</v>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 356.54 (CDF 0.997, 100.3% developed). CDF &lt;1.0 signals marginal reopens. Reported IE (337.54) shows negative IBNR (-20.07); disqualifies case adequacy assumption. Reported CL is primary. BF shows minor negative (-1.02). Reported CL selected as most credible method.</t>
         </is>
       </c>
-      <c r="I20" s="6" t="n">
+      <c r="I20" s="5" t="n">
         <v>356.54</v>
       </c>
-      <c r="J20" s="7" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Nearly mature (CDF 0.9970, 71 months); CL ultimate of 356.54 with slight negative IBNR (-1.07). IE method negative IBNR (-20.07) suggests reported count overstatement; CL is credible anchor.</t>
         </is>
       </c>
-      <c r="K20" s="8" t="n"/>
-      <c r="L20" s="9" t="n"/>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2784,21 +2769,21 @@
       <c r="G21" s="4" t="n">
         <v>369.4</v>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 369.40 (CDF 0.9962, 100.4% developed). CDF &lt;1.0 indicates reopens. Reported IE (358.12) shows negative IBNR (-12.69); case adequacy fails. Reported CL is primary. BF shows minor negative (-1.36). At near-full maturity, Reported CL is most reliable.</t>
         </is>
       </c>
-      <c r="I21" s="6" t="n">
+      <c r="I21" s="5" t="n">
         <v>369.4</v>
       </c>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="J21" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Nearly mature (CDF 0.9962, 59 months); CL ultimate of 369.40 with small negative IBNR (-1.41). Methods show modest development remaining; CL reflects current maturity.</t>
         </is>
       </c>
-      <c r="K21" s="8" t="n"/>
-      <c r="L21" s="9" t="n"/>
+      <c r="K21" s="6" t="n"/>
+      <c r="L21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2826,21 +2811,21 @@
       <c r="G22" s="4" t="n">
         <v>328.65</v>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 328.65 (CDF 0.9962, 100.4% developed). CDF &lt;1.0 indicates reopens. Reported IE (360.11) shows +30.21 IBNR (9.2% adjustment); plausibility questionable at near-full development. Reported CL is primary. BF shows minor negative (-1.37). CL selected.</t>
         </is>
       </c>
-      <c r="I22" s="6" t="n">
+      <c r="I22" s="5" t="n">
         <v>328.65</v>
       </c>
-      <c r="J22" s="7" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Nearly mature (CDF 0.9962, 47 months); CL ultimate of 328.65 with negative IBNR (-1.25). IE method shows IBNR of 30.21; CL reflects lower developmental pattern and is credible.</t>
         </is>
       </c>
-      <c r="K22" s="8" t="n"/>
-      <c r="L22" s="9" t="n"/>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2868,21 +2853,21 @@
       <c r="G23" s="4" t="n">
         <v>297.34</v>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 297.34 (CDF 0.9970, 100.3% developed). CDF &lt;1.0 marginal. Reported IE (339.98) shows +41.75 IBNR (14.0% adjustment); fitness weak at near-full development. Reported CL is primary. BF shows minor negative (-1.02). CL most credible at 48% developed.</t>
         </is>
       </c>
-      <c r="I23" s="6" t="n">
+      <c r="I23" s="5" t="n">
         <v>297.34</v>
       </c>
-      <c r="J23" s="7" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Developing (CDF 0.9970, 35 months); CL ultimate of 297.34 with slight negative IBNR (-0.89). IE method shows IBNR of 41.75; CL reflects reported count stability in early development.</t>
         </is>
       </c>
-      <c r="K23" s="8" t="n"/>
-      <c r="L23" s="9" t="n"/>
+      <c r="K23" s="6" t="n"/>
+      <c r="L23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2910,21 +2895,21 @@
       <c r="G24" s="4" t="n">
         <v>303.91</v>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 303.91 (CDF 0.9970, 100.3% developed). CDF &lt;1.0 marginal. Reported IE (317.43) shows +12.61 IBNR (4.1% adjustment); marginal given 53% development. Reported CL is primary. BF shows minor negative (-0.95). CL selected as most data-driven method.</t>
         </is>
       </c>
-      <c r="I24" s="6" t="n">
+      <c r="I24" s="5" t="n">
         <v>303.91</v>
       </c>
-      <c r="J24" s="7" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Developing (CDF 0.9970, 23 months); CL ultimate of 303.91 with slight negative IBNR (-0.91). Methods cluster around 303-317 range; CL is credible for developing cohort.</t>
         </is>
       </c>
-      <c r="K24" s="8" t="n"/>
-      <c r="L24" s="9" t="n"/>
+      <c r="K24" s="6" t="n"/>
+      <c r="L24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2952,24 +2937,24 @@
       <c r="G25" s="4" t="n">
         <v>286.07</v>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>Reported Count selected. Reported CL ultimate of 285.35 (CDF 1.1146, 89.7% developed). High CDF indicates significant development ahead (10.3%). Reported IE (292.35) shows +36.35 IBNR (12.4% adjustment); fitness weak at very early stage. Reported BF (286.07) very close to CL (0.26% difference). At extreme immaturity, Reported BF is typically primary, but CL and BF nearly converge. Selected midpoint/BF (286.07) for very green period; CDF volatility at 11 months. BF slightly preferred for a priori credibility.</t>
         </is>
       </c>
-      <c r="I25" s="6" t="n">
+      <c r="I25" s="5" t="n">
         <v>285.35</v>
       </c>
-      <c r="J25" s="7" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>Reported Count, Chain Ladder. Early developing (CDF 1.1146, 11 months); CL ultimate of 285.35 with IBNR of 29.35. CDF greater than 1.0 suggests early development may reverse; CL provides credible estimate at this immature stage despite tail uncertainty.</t>
         </is>
       </c>
-      <c r="K25" s="8" t="n"/>
-      <c r="L25" s="9" t="n"/>
+      <c r="K25" s="6" t="n"/>
+      <c r="L25" s="6" t="n"/>
     </row>
     <row r="26"/>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>